<commit_message>
data driven testing with data provider by excel
</commit_message>
<xml_diff>
--- a/testData/userDetails.xlsx
+++ b/testData/userDetails.xlsx
@@ -5,15 +5,16 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Chamod Ganegoda\Documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Test Automation\Learning-Selenium-Data-Driven-Testing\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{B31A5670-D097-4521-AAE2-6E30C63A2040}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE5576E2-D6E0-4598-9F0B-D010985C84C8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{64507181-7DE2-401F-ADF8-E81CB26BEF60}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -89,27 +90,12 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -118,8 +104,8 @@
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -500,4 +486,13 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB734CF0-3B40-4D2C-8A0B-FE64DE0712C5}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>